<commit_message>
agrego de inventario con su tabla en la base de datos y modificacion en Euclides para hacerlo mas visual
</commit_message>
<xml_diff>
--- a/Proyecto_Final_SemestreII/algoritmos/transacciones_ventas/proyecto.xlsx
+++ b/Proyecto_Final_SemestreII/algoritmos/transacciones_ventas/proyecto.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inventario" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +442,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Churrasco Waldemar</t>
+          <t>Negreira</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -482,6 +483,116 @@
         <is>
           <t>Casa de Patata</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Existencia</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0265</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Coca Cola</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CocaColaCompany</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3698</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pepsi 500 ml</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>200</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PepsiCola</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1235</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monster Ultra White</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>365</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Monster Energy</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>